<commit_message>
Deployed 5ce1c95c to dev with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/dev/assets/coremeta4cat_vocabulary.xlsx
+++ b/dev/assets/coremeta4cat_vocabulary.xlsx
@@ -1711,7 +1711,7 @@
       <c r="H10" s="13" t="inlineStr"/>
       <c r="I10" s="13" t="inlineStr">
         <is>
-          <t>CHEBI:52717</t>
+          <t>VOC4CAT:0007794</t>
         </is>
       </c>
       <c r="J10" s="13" t="inlineStr">
@@ -1906,7 +1906,7 @@
       <c r="H15" s="13" t="inlineStr"/>
       <c r="I15" s="13" t="inlineStr">
         <is>
-          <t>OBI:0000272</t>
+          <t>VOC4CAT:0007016</t>
         </is>
       </c>
       <c r="J15" s="13" t="inlineStr">
@@ -2076,7 +2076,7 @@
       <c r="H19" s="13" t="inlineStr"/>
       <c r="I19" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J19" s="13" t="inlineStr">
@@ -2168,7 +2168,7 @@
       <c r="H21" s="12" t="inlineStr"/>
       <c r="I21" s="12" t="inlineStr">
         <is>
-          <t>coremeta4cat:drying_device</t>
+          <t>VOC4CAT:0008122</t>
         </is>
       </c>
       <c r="J21" s="12" t="inlineStr">
@@ -2208,7 +2208,7 @@
       <c r="H22" s="12" t="inlineStr"/>
       <c r="I22" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008207</t>
         </is>
       </c>
       <c r="J22" s="12" t="inlineStr">
@@ -2248,7 +2248,7 @@
       <c r="H23" s="12" t="inlineStr"/>
       <c r="I23" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008206</t>
         </is>
       </c>
       <c r="J23" s="12" t="inlineStr">
@@ -2284,7 +2284,7 @@
       <c r="H24" s="13" t="inlineStr"/>
       <c r="I24" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J24" s="13" t="inlineStr">
@@ -2332,7 +2332,7 @@
       <c r="H25" s="12" t="inlineStr"/>
       <c r="I25" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008208</t>
         </is>
       </c>
       <c r="J25" s="12" t="inlineStr">
@@ -2592,7 +2592,7 @@
       <c r="H32" s="12" t="inlineStr"/>
       <c r="I32" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0000060</t>
         </is>
       </c>
       <c r="J32" s="12" t="inlineStr">
@@ -2628,7 +2628,7 @@
       <c r="H33" s="13" t="inlineStr"/>
       <c r="I33" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J33" s="13" t="inlineStr">
@@ -2833,7 +2833,7 @@
       <c r="H38" s="13" t="inlineStr"/>
       <c r="I38" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008116</t>
         </is>
       </c>
       <c r="J38" s="13" t="inlineStr">
@@ -2873,7 +2873,7 @@
       <c r="H39" s="12" t="inlineStr"/>
       <c r="I39" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0000056</t>
         </is>
       </c>
       <c r="J39" s="12" t="inlineStr">
@@ -3210,7 +3210,7 @@
       <c r="H48" s="13" t="inlineStr"/>
       <c r="I48" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J48" s="13" t="inlineStr">
@@ -3462,7 +3462,7 @@
       <c r="H54" s="12" t="inlineStr"/>
       <c r="I54" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008204</t>
         </is>
       </c>
       <c r="J54" s="12" t="inlineStr">
@@ -3498,7 +3498,7 @@
       <c r="H55" s="13" t="inlineStr"/>
       <c r="I55" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J55" s="13" t="inlineStr">
@@ -3542,7 +3542,7 @@
       <c r="H56" s="12" t="inlineStr"/>
       <c r="I56" s="12" t="inlineStr">
         <is>
-          <t>coremeta4cat:drying_device</t>
+          <t>VOC4CAT:0008122</t>
         </is>
       </c>
       <c r="J56" s="12" t="inlineStr">
@@ -3582,7 +3582,7 @@
       <c r="H57" s="12" t="inlineStr"/>
       <c r="I57" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008207</t>
         </is>
       </c>
       <c r="J57" s="12" t="inlineStr">
@@ -3622,7 +3622,7 @@
       <c r="H58" s="12" t="inlineStr"/>
       <c r="I58" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008206</t>
         </is>
       </c>
       <c r="J58" s="12" t="inlineStr">
@@ -3670,7 +3670,7 @@
       <c r="H59" s="12" t="inlineStr"/>
       <c r="I59" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008208</t>
         </is>
       </c>
       <c r="J59" s="12" t="inlineStr">
@@ -3751,7 +3751,7 @@
       <c r="H61" s="12" t="inlineStr"/>
       <c r="I61" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0000060</t>
         </is>
       </c>
       <c r="J61" s="12" t="inlineStr">
@@ -3923,7 +3923,7 @@
       <c r="H65" s="12" t="inlineStr"/>
       <c r="I65" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0000056</t>
         </is>
       </c>
       <c r="J65" s="12" t="inlineStr">
@@ -4044,7 +4044,7 @@
       <c r="H68" s="12" t="inlineStr"/>
       <c r="I68" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008204</t>
         </is>
       </c>
       <c r="J68" s="12" t="inlineStr">
@@ -4176,7 +4176,7 @@
       <c r="H71" s="12" t="inlineStr"/>
       <c r="I71" s="12" t="inlineStr">
         <is>
-          <t>coremeta4cat:drying_device</t>
+          <t>VOC4CAT:0008122</t>
         </is>
       </c>
       <c r="J71" s="12" t="inlineStr">
@@ -4216,7 +4216,7 @@
       <c r="H72" s="12" t="inlineStr"/>
       <c r="I72" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008207</t>
         </is>
       </c>
       <c r="J72" s="12" t="inlineStr">
@@ -4256,7 +4256,7 @@
       <c r="H73" s="12" t="inlineStr"/>
       <c r="I73" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008206</t>
         </is>
       </c>
       <c r="J73" s="12" t="inlineStr">
@@ -4304,7 +4304,7 @@
       <c r="H74" s="12" t="inlineStr"/>
       <c r="I74" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008208</t>
         </is>
       </c>
       <c r="J74" s="12" t="inlineStr">
@@ -4433,7 +4433,7 @@
       <c r="H77" s="12" t="inlineStr"/>
       <c r="I77" s="12" t="inlineStr">
         <is>
-          <t>coremeta4cat:stirrer_type</t>
+          <t>VOC4CAT:0008113</t>
         </is>
       </c>
       <c r="J77" s="12" t="inlineStr">
@@ -4517,7 +4517,7 @@
       <c r="H79" s="13" t="inlineStr"/>
       <c r="I79" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008116</t>
         </is>
       </c>
       <c r="J79" s="13" t="inlineStr">
@@ -4649,7 +4649,7 @@
       <c r="H82" s="13" t="inlineStr"/>
       <c r="I82" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J82" s="13" t="inlineStr">
@@ -4782,7 +4782,7 @@
       <c r="H85" s="12" t="inlineStr"/>
       <c r="I85" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J85" s="12" t="inlineStr">
@@ -5068,7 +5068,7 @@
       <c r="H92" s="13" t="inlineStr"/>
       <c r="I92" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J92" s="13" t="inlineStr">
@@ -5308,7 +5308,7 @@
       <c r="H97" s="12" t="inlineStr"/>
       <c r="I97" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J97" s="12" t="inlineStr">
@@ -5761,7 +5761,7 @@
       <c r="H107" s="12" t="inlineStr"/>
       <c r="I107" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J107" s="12" t="inlineStr">
@@ -6248,7 +6248,7 @@
       <c r="H118" s="13" t="inlineStr"/>
       <c r="I118" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J118" s="13" t="inlineStr">
@@ -6692,7 +6692,7 @@
       <c r="H129" s="12" t="inlineStr"/>
       <c r="I129" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008204</t>
         </is>
       </c>
       <c r="J129" s="12" t="inlineStr">
@@ -6736,7 +6736,7 @@
       <c r="H130" s="12" t="inlineStr"/>
       <c r="I130" s="12" t="inlineStr">
         <is>
-          <t>coremeta4cat:drying_device</t>
+          <t>VOC4CAT:0008122</t>
         </is>
       </c>
       <c r="J130" s="12" t="inlineStr">
@@ -6776,7 +6776,7 @@
       <c r="H131" s="12" t="inlineStr"/>
       <c r="I131" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008207</t>
         </is>
       </c>
       <c r="J131" s="12" t="inlineStr">
@@ -6816,7 +6816,7 @@
       <c r="H132" s="12" t="inlineStr"/>
       <c r="I132" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008206</t>
         </is>
       </c>
       <c r="J132" s="12" t="inlineStr">
@@ -6864,7 +6864,7 @@
       <c r="H133" s="12" t="inlineStr"/>
       <c r="I133" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008208</t>
         </is>
       </c>
       <c r="J133" s="12" t="inlineStr">
@@ -6945,7 +6945,7 @@
       <c r="H135" s="12" t="inlineStr"/>
       <c r="I135" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0000060</t>
         </is>
       </c>
       <c r="J135" s="12" t="inlineStr">
@@ -7117,7 +7117,7 @@
       <c r="H139" s="12" t="inlineStr"/>
       <c r="I139" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0000056</t>
         </is>
       </c>
       <c r="J139" s="12" t="inlineStr">
@@ -7442,7 +7442,7 @@
       <c r="H146" s="12" t="inlineStr"/>
       <c r="I146" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J146" s="12" t="inlineStr">
@@ -7651,7 +7651,7 @@
       <c r="H151" s="12" t="inlineStr"/>
       <c r="I151" s="12" t="inlineStr">
         <is>
-          <t>coremeta4cat:drying_device</t>
+          <t>VOC4CAT:0008122</t>
         </is>
       </c>
       <c r="J151" s="12" t="inlineStr">
@@ -7691,7 +7691,7 @@
       <c r="H152" s="12" t="inlineStr"/>
       <c r="I152" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008207</t>
         </is>
       </c>
       <c r="J152" s="12" t="inlineStr">
@@ -7731,7 +7731,7 @@
       <c r="H153" s="12" t="inlineStr"/>
       <c r="I153" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008206</t>
         </is>
       </c>
       <c r="J153" s="12" t="inlineStr">
@@ -7779,7 +7779,7 @@
       <c r="H154" s="12" t="inlineStr"/>
       <c r="I154" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008208</t>
         </is>
       </c>
       <c r="J154" s="12" t="inlineStr">
@@ -7860,7 +7860,7 @@
       <c r="H156" s="12" t="inlineStr"/>
       <c r="I156" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0000060</t>
         </is>
       </c>
       <c r="J156" s="12" t="inlineStr">
@@ -8032,7 +8032,7 @@
       <c r="H160" s="12" t="inlineStr"/>
       <c r="I160" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0000056</t>
         </is>
       </c>
       <c r="J160" s="12" t="inlineStr">
@@ -9058,7 +9058,7 @@
       <c r="H183" s="12" t="inlineStr"/>
       <c r="I183" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J183" s="12" t="inlineStr">
@@ -9335,7 +9335,7 @@
       <c r="H189" s="12" t="inlineStr"/>
       <c r="I189" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J189" s="12" t="inlineStr">
@@ -9536,7 +9536,7 @@
       <c r="H194" s="13" t="inlineStr"/>
       <c r="I194" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J194" s="13" t="inlineStr">
@@ -9828,7 +9828,7 @@
       <c r="H201" s="12" t="inlineStr"/>
       <c r="I201" s="12" t="inlineStr">
         <is>
-          <t>coremeta4cat:precipitation_agent</t>
+          <t>VOC4CAT:0008203</t>
         </is>
       </c>
       <c r="J201" s="12" t="inlineStr">
@@ -10060,7 +10060,7 @@
       <c r="H206" s="12" t="inlineStr"/>
       <c r="I206" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J206" s="12" t="inlineStr">
@@ -10104,7 +10104,7 @@
       <c r="H207" s="12" t="inlineStr"/>
       <c r="I207" s="12" t="inlineStr">
         <is>
-          <t>coremeta4cat:drying_device</t>
+          <t>VOC4CAT:0008122</t>
         </is>
       </c>
       <c r="J207" s="12" t="inlineStr">
@@ -10144,7 +10144,7 @@
       <c r="H208" s="12" t="inlineStr"/>
       <c r="I208" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008207</t>
         </is>
       </c>
       <c r="J208" s="12" t="inlineStr">
@@ -10184,7 +10184,7 @@
       <c r="H209" s="12" t="inlineStr"/>
       <c r="I209" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008206</t>
         </is>
       </c>
       <c r="J209" s="12" t="inlineStr">
@@ -10232,7 +10232,7 @@
       <c r="H210" s="12" t="inlineStr"/>
       <c r="I210" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008208</t>
         </is>
       </c>
       <c r="J210" s="12" t="inlineStr">
@@ -10350,7 +10350,7 @@
       <c r="H213" s="12" t="inlineStr"/>
       <c r="I213" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0000060</t>
         </is>
       </c>
       <c r="J213" s="12" t="inlineStr">
@@ -10522,7 +10522,7 @@
       <c r="H217" s="12" t="inlineStr"/>
       <c r="I217" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0000056</t>
         </is>
       </c>
       <c r="J217" s="12" t="inlineStr">
@@ -11270,7 +11270,7 @@
       <c r="H18" s="12" t="inlineStr"/>
       <c r="I18" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J18" s="12" t="inlineStr">
@@ -11536,7 +11536,7 @@
       <c r="H25" s="13" t="inlineStr"/>
       <c r="I25" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J25" s="13" t="inlineStr">
@@ -12490,7 +12490,7 @@
       <c r="H48" s="13" t="inlineStr"/>
       <c r="I48" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J48" s="13" t="inlineStr">
@@ -12882,7 +12882,7 @@
       <c r="H57" s="12" t="inlineStr"/>
       <c r="I57" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J57" s="12" t="inlineStr">
@@ -13215,7 +13215,7 @@
       <c r="H65" s="13" t="inlineStr"/>
       <c r="I65" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J65" s="13" t="inlineStr">
@@ -13681,7 +13681,7 @@
       <c r="H76" s="12" t="inlineStr"/>
       <c r="I76" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J76" s="12" t="inlineStr">
@@ -13814,7 +13814,7 @@
       <c r="H79" s="12" t="inlineStr"/>
       <c r="I79" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J79" s="12" t="inlineStr">
@@ -14551,7 +14551,7 @@
       <c r="H97" s="13" t="inlineStr"/>
       <c r="I97" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J97" s="13" t="inlineStr">
@@ -14643,7 +14643,7 @@
       <c r="H99" s="12" t="inlineStr"/>
       <c r="I99" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J99" s="12" t="inlineStr">
@@ -15110,7 +15110,7 @@
       <c r="H110" s="12" t="inlineStr"/>
       <c r="I110" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J110" s="12" t="inlineStr">
@@ -15762,7 +15762,7 @@
       <c r="H125" s="12" t="inlineStr"/>
       <c r="I125" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J125" s="12" t="inlineStr">
@@ -16056,7 +16056,7 @@
       <c r="H132" s="13" t="inlineStr"/>
       <c r="I132" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008116</t>
         </is>
       </c>
       <c r="J132" s="13" t="inlineStr">
@@ -18763,7 +18763,7 @@
       <c r="H195" s="12" t="inlineStr"/>
       <c r="I195" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J195" s="12" t="inlineStr">
@@ -19283,7 +19283,7 @@
       <c r="H207" s="12" t="inlineStr"/>
       <c r="I207" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J207" s="12" t="inlineStr">
@@ -19807,7 +19807,7 @@
       <c r="H220" s="13" t="inlineStr"/>
       <c r="I220" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J220" s="13" t="inlineStr">
@@ -20625,7 +20625,7 @@
       <c r="H239" s="13" t="inlineStr"/>
       <c r="I239" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008116</t>
         </is>
       </c>
       <c r="J239" s="13" t="inlineStr">
@@ -21962,10 +21962,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
@@ -22122,7 +22122,7 @@
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>catalyst type</t>
+          <t>has catalyst type</t>
         </is>
       </c>
       <c r="B4" s="10" t="inlineStr">
@@ -22138,7 +22138,7 @@
       </c>
       <c r="E4" s="10" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>CatalystType</t>
         </is>
       </c>
       <c r="F4" s="10" t="inlineStr">
@@ -22146,7 +22146,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G4" s="10" t="inlineStr"/>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="H4" s="10" t="inlineStr"/>
       <c r="I4" s="10" t="inlineStr">
         <is>
@@ -22161,55 +22165,46 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>reactor temperature range</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C5" s="12" t="inlineStr"/>
-      <c r="D5" s="12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>QuantitativeRange</t>
-        </is>
-      </c>
-      <c r="F5" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G5" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H5" s="12" t="inlineStr"/>
-      <c r="I5" s="12" t="inlineStr">
-        <is>
-          <t>VOC4CAT:0007032</t>
-        </is>
-      </c>
-      <c r="J5" s="12" t="inlineStr">
-        <is>
-          <t>Temperature range in the reactor during the reaction, provided as a
-QuantitativeRange with min_value and max_value (unit_code: "Cel").
-For a single set-point, set min_value equal to max_value.</t>
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>CatalystType</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>has catalyst type</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr"/>
+      <c r="F5" s="13" t="inlineStr"/>
+      <c r="G5" s="13" t="inlineStr"/>
+      <c r="H5" s="13" t="inlineStr"/>
+      <c r="I5" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0007014</t>
+        </is>
+      </c>
+      <c r="J5" s="13" t="inlineStr">
+        <is>
+          <t>Type of catalyst used (e.g. heterogeneous, homogeneous, biocatalyst).
+For heterogeneous catalysts, use voc4cat terms where available.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
         <is>
-          <t>QuantitativeRange</t>
+          <t>HeterogeneousCatalyst</t>
         </is>
       </c>
       <c r="B6" s="13" t="inlineStr">
@@ -22219,12 +22214,12 @@
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>reactor temperature range</t>
+          <t>CatalystType</t>
         </is>
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>R</t>
         </is>
       </c>
       <c r="E6" s="13" t="inlineStr"/>
@@ -22233,10 +22228,888 @@
       <c r="H6" s="13" t="inlineStr"/>
       <c r="I6" s="13" t="inlineStr">
         <is>
+          <t>VOC4CAT:0007003</t>
+        </is>
+      </c>
+      <c r="J6" s="13" t="inlineStr">
+        <is>
+          <t>A substance that increases the rate of a chemical reaction that is in a different phase than the reagents.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>HomogeneousCatalyst</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>CatalystType</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr"/>
+      <c r="F7" s="13" t="inlineStr"/>
+      <c r="G7" s="13" t="inlineStr"/>
+      <c r="H7" s="13" t="inlineStr"/>
+      <c r="I7" s="13" t="inlineStr">
+        <is>
+          <t>coremeta4cat:HomogeneousCatalyst</t>
+        </is>
+      </c>
+      <c r="J7" s="13" t="inlineStr">
+        <is>
+          <t>A substance that increses the rate of a chemical reaction that is in the same phase as the reagents.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>BioCatalyst</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>CatalystType</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr"/>
+      <c r="F8" s="13" t="inlineStr"/>
+      <c r="G8" s="13" t="inlineStr"/>
+      <c r="H8" s="13" t="inlineStr"/>
+      <c r="I8" s="13" t="inlineStr">
+        <is>
+          <t>coremeta4cat:BioCatalyst</t>
+        </is>
+      </c>
+      <c r="J8" s="13" t="inlineStr">
+        <is>
+          <t>An enzyme or cell that catalyzes a biocatalytic reaction. Subclass of Catalyst (AgenticEntity). The physical form in which it is applied is described by an associated BiocatalystPreparation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>ElectroCatalyst</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>CatalystType</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr"/>
+      <c r="F9" s="13" t="inlineStr"/>
+      <c r="G9" s="13" t="inlineStr"/>
+      <c r="H9" s="13" t="inlineStr"/>
+      <c r="I9" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0000255</t>
+        </is>
+      </c>
+      <c r="J9" s="13" t="inlineStr">
+        <is>
+          <t>The characteristics of a material or substance that determine how it interacts or responds to a magnetic field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>ThinFilmCatalyst</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>CatalystType</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr"/>
+      <c r="F10" s="13" t="inlineStr"/>
+      <c r="G10" s="13" t="inlineStr"/>
+      <c r="H10" s="13" t="inlineStr"/>
+      <c r="I10" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0000019</t>
+        </is>
+      </c>
+      <c r="J10" s="13" t="inlineStr">
+        <is>
+          <t>A catalyst introduced to the reaction chamber in the form of a thin film. To form a thin film, a (powdered) catalyst is deposited on a substrate (e.g., glass or metal) using an appropriate deposition technique.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>BulkCatalyst</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>CatalystType</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr"/>
+      <c r="F11" s="13" t="inlineStr"/>
+      <c r="G11" s="13" t="inlineStr"/>
+      <c r="H11" s="13" t="inlineStr"/>
+      <c r="I11" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0007015</t>
+        </is>
+      </c>
+      <c r="J11" s="13" t="inlineStr">
+        <is>
+          <t>A catalyst that consists mainly of the active ingredient or phase.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>PowerderedCatalyst</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>CatalystType</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr"/>
+      <c r="F12" s="13" t="inlineStr"/>
+      <c r="G12" s="13" t="inlineStr"/>
+      <c r="H12" s="13" t="inlineStr"/>
+      <c r="I12" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0000017</t>
+        </is>
+      </c>
+      <c r="J12" s="13" t="inlineStr">
+        <is>
+          <t>A catalyst introduced to the reaction chamber in the form of a powder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>DepositedSampleCatalyst</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>CatalystType</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr"/>
+      <c r="F13" s="13" t="inlineStr"/>
+      <c r="G13" s="13" t="inlineStr"/>
+      <c r="H13" s="13" t="inlineStr"/>
+      <c r="I13" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0000038</t>
+        </is>
+      </c>
+      <c r="J13" s="13" t="inlineStr">
+        <is>
+          <t>A thin film of the catalyst deposited on an appropriate for the application substrate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>PhotoCatalyst</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>CatalystType</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E14" s="13" t="inlineStr"/>
+      <c r="F14" s="13" t="inlineStr"/>
+      <c r="G14" s="13" t="inlineStr"/>
+      <c r="H14" s="13" t="inlineStr"/>
+      <c r="I14" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0000002</t>
+        </is>
+      </c>
+      <c r="J14" s="13" t="inlineStr">
+        <is>
+          <t>A material that absorbs photons (light) of appropriate energy and initiates or accelerates a photochemical reaction, while it regenerates itself after each reaction cycle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>SupportedCatalsyt</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>CatalystType</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="inlineStr"/>
+      <c r="F15" s="13" t="inlineStr"/>
+      <c r="G15" s="13" t="inlineStr"/>
+      <c r="H15" s="13" t="inlineStr"/>
+      <c r="I15" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0007034</t>
+        </is>
+      </c>
+      <c r="J15" s="13" t="inlineStr">
+        <is>
+          <t>A catalyst where the active material is usually the minority phase and fixed on a high surface area, relatively inert solid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>has reaction type</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr"/>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>ReactionType</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="inlineStr"/>
+      <c r="H16" s="10" t="inlineStr"/>
+      <c r="I16" s="10" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0007010</t>
+        </is>
+      </c>
+      <c r="J16" s="10" t="inlineStr">
+        <is>
+          <t>A group of chemical reactions with common conditions or reactants, e.g. Oxidation, Hydrogenation, Reduction, Cracking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>ReactionType</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>has reaction type</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E17" s="13" t="inlineStr"/>
+      <c r="F17" s="13" t="inlineStr"/>
+      <c r="G17" s="13" t="inlineStr"/>
+      <c r="H17" s="13" t="inlineStr"/>
+      <c r="I17" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0007010</t>
+        </is>
+      </c>
+      <c r="J17" s="13" t="inlineStr">
+        <is>
+          <t>A group of chemical reactions with common conditions or reactants, e.g. Oxidation, Hydrogenation, Reduction, Cracking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>Hydrogenation</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>ReactionType</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E18" s="13" t="inlineStr"/>
+      <c r="F18" s="13" t="inlineStr"/>
+      <c r="G18" s="13" t="inlineStr"/>
+      <c r="H18" s="13" t="inlineStr"/>
+      <c r="I18" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0000260</t>
+        </is>
+      </c>
+      <c r="J18" s="13" t="inlineStr">
+        <is>
+          <t>A chemical reaction of molecular hydrogen (H2) and another chemical species, typically facilitated by a catalyst.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>CarbonDioxideHydrogenation</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="inlineStr">
+        <is>
+          <t>ReactionType</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E19" s="13" t="inlineStr"/>
+      <c r="F19" s="13" t="inlineStr"/>
+      <c r="G19" s="13" t="inlineStr"/>
+      <c r="H19" s="13" t="inlineStr"/>
+      <c r="I19" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0000259</t>
+        </is>
+      </c>
+      <c r="J19" s="13" t="inlineStr">
+        <is>
+          <t>The reaction of carbon dioxide (CO2) with molecular hydrogen (H2) to produce value-added hydrocarbons or alcohols.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>Oxidation</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>ReactionType</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E20" s="13" t="inlineStr"/>
+      <c r="F20" s="13" t="inlineStr"/>
+      <c r="G20" s="13" t="inlineStr"/>
+      <c r="H20" s="13" t="inlineStr"/>
+      <c r="I20" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0000097</t>
+        </is>
+      </c>
+      <c r="J20" s="13" t="inlineStr">
+        <is>
+          <t>The loss of electrons or an increase in the oxidation state of a species.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>SelectiveOxidation</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>ReactionType</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E21" s="13" t="inlineStr"/>
+      <c r="F21" s="13" t="inlineStr"/>
+      <c r="G21" s="13" t="inlineStr"/>
+      <c r="H21" s="13" t="inlineStr"/>
+      <c r="I21" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0000261</t>
+        </is>
+      </c>
+      <c r="J21" s="13" t="inlineStr">
+        <is>
+          <t>The targeted oxidation of a specific bond or functional group in a molecule leaving other sites unaffected, often directed by a catalyst.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>CarbonMonoxideOxidation</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C22" s="13" t="inlineStr">
+        <is>
+          <t>ReactionType</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E22" s="13" t="inlineStr"/>
+      <c r="F22" s="13" t="inlineStr"/>
+      <c r="G22" s="13" t="inlineStr"/>
+      <c r="H22" s="13" t="inlineStr"/>
+      <c r="I22" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0000289</t>
+        </is>
+      </c>
+      <c r="J22" s="13" t="inlineStr">
+        <is>
+          <t>The reaction in which carbon monoxide (CO) is converted to carbon dioxide (CO2) through interaction with an oxidizing agent, typically oxygen (O2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>Dehydrogenation</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>ReactionType</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E23" s="13" t="inlineStr"/>
+      <c r="F23" s="13" t="inlineStr"/>
+      <c r="G23" s="13" t="inlineStr"/>
+      <c r="H23" s="13" t="inlineStr"/>
+      <c r="I23" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0000297</t>
+        </is>
+      </c>
+      <c r="J23" s="13" t="inlineStr">
+        <is>
+          <t>A chemical reaction that involves the removal of two or more hydrogen atoms from a molecule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>CarbonCouplingReaction</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C24" s="13" t="inlineStr">
+        <is>
+          <t>ReactionType</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E24" s="13" t="inlineStr"/>
+      <c r="F24" s="13" t="inlineStr"/>
+      <c r="G24" s="13" t="inlineStr"/>
+      <c r="H24" s="13" t="inlineStr"/>
+      <c r="I24" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0000223</t>
+        </is>
+      </c>
+      <c r="J24" s="13" t="inlineStr">
+        <is>
+          <t>A chemical reaction where a carbon-carbon bond is formed from two carbon-containing fragments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>Hydrodeoxygenation</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>ReactionType</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="inlineStr"/>
+      <c r="F25" s="13" t="inlineStr"/>
+      <c r="G25" s="13" t="inlineStr"/>
+      <c r="H25" s="13" t="inlineStr"/>
+      <c r="I25" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0000226</t>
+        </is>
+      </c>
+      <c r="J25" s="13" t="inlineStr">
+        <is>
+          <t>A catalytic process in which oxygen is removed from oxygenated organic compounds using hydrogen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>OxygenEvolutionReaction</t>
+        </is>
+      </c>
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C26" s="13" t="inlineStr">
+        <is>
+          <t>ReactionType</t>
+        </is>
+      </c>
+      <c r="D26" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E26" s="13" t="inlineStr"/>
+      <c r="F26" s="13" t="inlineStr"/>
+      <c r="G26" s="13" t="inlineStr"/>
+      <c r="H26" s="13" t="inlineStr"/>
+      <c r="I26" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0000236</t>
+        </is>
+      </c>
+      <c r="J26" s="13" t="inlineStr">
+        <is>
+          <t>A chemical reaction of generating molecular oxygen in electrochemistry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>Hydroxylation</t>
+        </is>
+      </c>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C27" s="13" t="inlineStr">
+        <is>
+          <t>ReactionType</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E27" s="13" t="inlineStr"/>
+      <c r="F27" s="13" t="inlineStr"/>
+      <c r="G27" s="13" t="inlineStr"/>
+      <c r="H27" s="13" t="inlineStr"/>
+      <c r="I27" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0000258</t>
+        </is>
+      </c>
+      <c r="J27" s="13" t="inlineStr">
+        <is>
+          <t>The addition of a hydroxyl group (-OH) to a molecule, typically by replacing a hydrogen atom.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>FischerTropschSynthesis</t>
+        </is>
+      </c>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>ReactionType</t>
+        </is>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E28" s="13" t="inlineStr"/>
+      <c r="F28" s="13" t="inlineStr"/>
+      <c r="G28" s="13" t="inlineStr"/>
+      <c r="H28" s="13" t="inlineStr"/>
+      <c r="I28" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0000280</t>
+        </is>
+      </c>
+      <c r="J28" s="13" t="inlineStr">
+        <is>
+          <t>A catalytic chemical reaction in which a mixture of carbon monoxide (CO) and hydrogen (H2), is converted via a chain-growth mechanism into long-chain hydrocarbons (e.g., alkanes, alkenes or alcohols)—typically using iron or cobalt catalysts under moderate to high pressures and temperatures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>reactor temperature range</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr"/>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>QuantitativeRange</t>
+        </is>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G29" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H29" s="12" t="inlineStr"/>
+      <c r="I29" s="12" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0007032</t>
+        </is>
+      </c>
+      <c r="J29" s="12" t="inlineStr">
+        <is>
+          <t>Temperature range in the reactor during the reaction, provided as a
+QuantitativeRange with min_value and max_value (unit_code: "Cel").
+For a single set-point, set min_value equal to max_value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>QuantitativeRange</t>
+        </is>
+      </c>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C30" s="13" t="inlineStr">
+        <is>
+          <t>reactor temperature range</t>
+        </is>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E30" s="13" t="inlineStr"/>
+      <c r="F30" s="13" t="inlineStr"/>
+      <c r="G30" s="13" t="inlineStr"/>
+      <c r="H30" s="13" t="inlineStr"/>
+      <c r="I30" s="13" t="inlineStr">
+        <is>
           <t>qudt:Quantity</t>
         </is>
       </c>
-      <c r="J6" s="13" t="inlineStr">
+      <c r="J30" s="13" t="inlineStr">
         <is>
           <t>A quantitative property expressed as a range between a lower and upper bound,
 sharing a common unit. Used where an experiment operates over a range of
@@ -22247,271 +23120,271 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C7" s="12" t="inlineStr">
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
         <is>
           <t>QuantitativeRange</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E7" s="12" t="inlineStr">
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E31" s="12" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="F7" s="12" t="inlineStr"/>
-      <c r="G7" s="12" t="inlineStr"/>
-      <c r="H7" s="12" t="inlineStr"/>
-      <c r="I7" s="12" t="inlineStr"/>
-      <c r="J7" s="12" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="F31" s="12" t="inlineStr"/>
+      <c r="G31" s="12" t="inlineStr"/>
+      <c r="H31" s="12" t="inlineStr"/>
+      <c r="I31" s="12" t="inlineStr"/>
+      <c r="J31" s="12" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
         <is>
           <t>QuantitativeRange</t>
         </is>
       </c>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E32" s="12" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="F8" s="12" t="inlineStr"/>
-      <c r="G8" s="12" t="inlineStr"/>
-      <c r="H8" s="12" t="inlineStr"/>
-      <c r="I8" s="12" t="inlineStr"/>
-      <c r="J8" s="12" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="F32" s="12" t="inlineStr"/>
+      <c r="G32" s="12" t="inlineStr"/>
+      <c r="H32" s="12" t="inlineStr"/>
+      <c r="I32" s="12" t="inlineStr"/>
+      <c r="J32" s="12" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
         <is>
           <t>has atmosphere</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="inlineStr"/>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="inlineStr">
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="inlineStr"/>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E33" s="12" t="inlineStr">
         <is>
           <t>Atmosphere</t>
         </is>
       </c>
-      <c r="F9" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G9" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H9" s="12" t="inlineStr"/>
-      <c r="I9" s="12" t="inlineStr">
-        <is>
-          <t>SIO:000008</t>
-        </is>
-      </c>
-      <c r="J9" s="12" t="inlineStr">
+      <c r="F33" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G33" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H33" s="12" t="inlineStr"/>
+      <c r="I33" s="12" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0007809</t>
+        </is>
+      </c>
+      <c r="J33" s="12" t="inlineStr">
         <is>
           <t>Gaseous environment or atmospheric conditions during a process.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="13" t="inlineStr">
         <is>
           <t>Atmosphere</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B34" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="C34" s="13" t="inlineStr">
         <is>
           <t>has atmosphere</t>
         </is>
       </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E10" s="13" t="inlineStr"/>
-      <c r="F10" s="13" t="inlineStr"/>
-      <c r="G10" s="13" t="inlineStr"/>
-      <c r="H10" s="13" t="inlineStr"/>
-      <c r="I10" s="13" t="inlineStr">
+      <c r="D34" s="13" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E34" s="13" t="inlineStr"/>
+      <c r="F34" s="13" t="inlineStr"/>
+      <c r="G34" s="13" t="inlineStr"/>
+      <c r="H34" s="13" t="inlineStr"/>
+      <c r="I34" s="13" t="inlineStr">
         <is>
           <t>coremeta4cat:Atmosphere</t>
         </is>
       </c>
-      <c r="J10" s="13" t="inlineStr">
+      <c r="J34" s="13" t="inlineStr">
         <is>
           <t>A qualitative descriptor of the gaseous environment or atmospheric
 conditions during a process (e.g. "air", "N2", "5% H2/Ar").</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
         <is>
           <t>CalcinationGaseousEnvironment</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C35" s="13" t="inlineStr">
         <is>
           <t>Atmosphere</t>
         </is>
       </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E11" s="13" t="inlineStr"/>
-      <c r="F11" s="13" t="inlineStr"/>
-      <c r="G11" s="13" t="inlineStr"/>
-      <c r="H11" s="13" t="inlineStr"/>
-      <c r="I11" s="13" t="inlineStr">
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E35" s="13" t="inlineStr"/>
+      <c r="F35" s="13" t="inlineStr"/>
+      <c r="G35" s="13" t="inlineStr"/>
+      <c r="H35" s="13" t="inlineStr"/>
+      <c r="I35" s="13" t="inlineStr">
         <is>
           <t>VOC4CAT:0000055</t>
         </is>
       </c>
-      <c r="J11" s="13" t="inlineStr">
+      <c r="J35" s="13" t="inlineStr">
         <is>
           <t>The specific gaseous environment maintained during a calcination step
 (e.g. "air", "N2", "10% O2/N2").</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
         <is>
           <t>experiment pressure</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C12" s="12" t="inlineStr"/>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E12" s="12" t="inlineStr">
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="inlineStr"/>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E36" s="12" t="inlineStr">
         <is>
           <t>Pressure</t>
         </is>
       </c>
-      <c r="F12" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G12" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H12" s="12" t="inlineStr"/>
-      <c r="I12" s="12" t="inlineStr">
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G36" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H36" s="12" t="inlineStr"/>
+      <c r="I36" s="12" t="inlineStr">
         <is>
           <t>VOC4CAT:0000118</t>
         </is>
       </c>
-      <c r="J12" s="12" t="inlineStr">
+      <c r="J36" s="12" t="inlineStr">
         <is>
           <t>Total pressure in the reactor during the experiment.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="12" t="inlineStr">
         <is>
           <t>feed composition range</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C13" s="12" t="inlineStr"/>
-      <c r="D13" s="12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E13" s="12" t="inlineStr">
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="inlineStr"/>
+      <c r="D37" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E37" s="12" t="inlineStr">
         <is>
           <t>QuantitativeRange</t>
         </is>
       </c>
-      <c r="F13" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G13" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H13" s="12" t="inlineStr"/>
-      <c r="I13" s="12" t="inlineStr">
+      <c r="F37" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G37" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H37" s="12" t="inlineStr"/>
+      <c r="I37" s="12" t="inlineStr">
         <is>
           <t>coremeta4cat:feed_composition_range</t>
         </is>
       </c>
-      <c r="J13" s="12" t="inlineStr">
+      <c r="J37" s="12" t="inlineStr">
         <is>
           <t>Feed composition range studied, provided as a QuantitativeRange.
 Express concentration bounds in an appropriate unit (e.g. "mol/L", "%" for
@@ -22519,37 +23392,37 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="13" t="inlineStr">
         <is>
           <t>QuantitativeRange</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B38" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="C38" s="13" t="inlineStr">
         <is>
           <t>feed composition range</t>
         </is>
       </c>
-      <c r="D14" s="13" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E14" s="13" t="inlineStr"/>
-      <c r="F14" s="13" t="inlineStr"/>
-      <c r="G14" s="13" t="inlineStr"/>
-      <c r="H14" s="13" t="inlineStr"/>
-      <c r="I14" s="13" t="inlineStr">
+      <c r="D38" s="13" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E38" s="13" t="inlineStr"/>
+      <c r="F38" s="13" t="inlineStr"/>
+      <c r="G38" s="13" t="inlineStr"/>
+      <c r="H38" s="13" t="inlineStr"/>
+      <c r="I38" s="13" t="inlineStr">
         <is>
           <t>qudt:Quantity</t>
         </is>
       </c>
-      <c r="J14" s="13" t="inlineStr">
+      <c r="J38" s="13" t="inlineStr">
         <is>
           <t>A quantitative property expressed as a range between a lower and upper bound,
 sharing a common unit. Used where an experiment operates over a range of
@@ -22560,117 +23433,117 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="12" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
         <is>
           <t>has experiment duration</t>
         </is>
       </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C15" s="12" t="inlineStr"/>
-      <c r="D15" s="12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E15" s="12" t="inlineStr">
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C39" s="12" t="inlineStr"/>
+      <c r="D39" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E39" s="12" t="inlineStr">
         <is>
           <t>Duration</t>
         </is>
       </c>
-      <c r="F15" s="12" t="inlineStr"/>
-      <c r="G15" s="12" t="inlineStr"/>
-      <c r="H15" s="12" t="inlineStr"/>
-      <c r="I15" s="12" t="inlineStr">
+      <c r="F39" s="12" t="inlineStr"/>
+      <c r="G39" s="12" t="inlineStr"/>
+      <c r="H39" s="12" t="inlineStr"/>
+      <c r="I39" s="12" t="inlineStr">
         <is>
           <t>SIO:000008</t>
         </is>
       </c>
-      <c r="J15" s="12" t="inlineStr">
+      <c r="J39" s="12" t="inlineStr">
         <is>
           <t>Total duration of the experiment or measurement run.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="13" t="inlineStr">
         <is>
           <t>Duration</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B40" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C16" s="13" t="inlineStr">
+      <c r="C40" s="13" t="inlineStr">
         <is>
           <t>has experiment duration</t>
         </is>
       </c>
-      <c r="D16" s="13" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E16" s="13" t="inlineStr"/>
-      <c r="F16" s="13" t="inlineStr"/>
-      <c r="G16" s="13" t="inlineStr"/>
-      <c r="H16" s="13" t="inlineStr"/>
-      <c r="I16" s="13" t="inlineStr">
-        <is>
-          <t>qudt:Quantity</t>
-        </is>
-      </c>
-      <c r="J16" s="13" t="inlineStr">
+      <c r="D40" s="13" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E40" s="13" t="inlineStr"/>
+      <c r="F40" s="13" t="inlineStr"/>
+      <c r="G40" s="13" t="inlineStr"/>
+      <c r="H40" s="13" t="inlineStr"/>
+      <c r="I40" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0008120</t>
+        </is>
+      </c>
+      <c r="J40" s="13" t="inlineStr">
         <is>
           <t>A quantitative measure of elapsed time (duration of a process step).</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="11" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="11" t="inlineStr">
         <is>
           <t>product identification method</t>
         </is>
       </c>
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="inlineStr"/>
-      <c r="D17" s="11" t="inlineStr">
+      <c r="B41" s="11" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="inlineStr"/>
+      <c r="D41" s="11" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E41" s="11" t="inlineStr">
         <is>
           <t>ProductIdentificationMethod</t>
         </is>
       </c>
-      <c r="F17" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G17" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H17" s="11" t="inlineStr"/>
-      <c r="I17" s="11" t="inlineStr">
+      <c r="F41" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G41" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H41" s="11" t="inlineStr"/>
+      <c r="I41" s="11" t="inlineStr">
         <is>
           <t>coremeta4cat:product_identification_method</t>
         </is>
       </c>
-      <c r="J17" s="11" t="inlineStr">
+      <c r="J41" s="11" t="inlineStr">
         <is>
           <t>The analytical method used to identify and/or quantify reaction products.
 Should reference a CharacterizationTechnique instance (e.g. GCMS, HPLC_MS).
@@ -22678,37 +23551,37 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="13" t="inlineStr">
         <is>
           <t>ProductIdentificationMethod</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B42" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C18" s="13" t="inlineStr">
+      <c r="C42" s="13" t="inlineStr">
         <is>
           <t>product identification method</t>
         </is>
       </c>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="D42" s="13" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E18" s="13" t="inlineStr"/>
-      <c r="F18" s="13" t="inlineStr"/>
-      <c r="G18" s="13" t="inlineStr"/>
-      <c r="H18" s="13" t="inlineStr"/>
-      <c r="I18" s="13" t="inlineStr">
+      <c r="E42" s="13" t="inlineStr"/>
+      <c r="F42" s="13" t="inlineStr"/>
+      <c r="G42" s="13" t="inlineStr"/>
+      <c r="H42" s="13" t="inlineStr"/>
+      <c r="I42" s="13" t="inlineStr">
         <is>
           <t>OBI:0000272</t>
         </is>
       </c>
-      <c r="J18" s="13" t="inlineStr">
+      <c r="J42" s="13" t="inlineStr">
         <is>
           <t>Abstract Plan representing the method used to identify and quantify reaction
 products. In practice, users should reference a concrete CharacterizationTechnique
@@ -22719,41 +23592,113 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="11" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="13" t="inlineStr">
+        <is>
+          <t>LiquidPhaseAnalysis</t>
+        </is>
+      </c>
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C43" s="13" t="inlineStr">
+        <is>
+          <t>ProductIdentificationMethod</t>
+        </is>
+      </c>
+      <c r="D43" s="13" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E43" s="13" t="inlineStr"/>
+      <c r="F43" s="13" t="inlineStr"/>
+      <c r="G43" s="13" t="inlineStr"/>
+      <c r="H43" s="13" t="inlineStr"/>
+      <c r="I43" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0007813</t>
+        </is>
+      </c>
+      <c r="J43" s="13" t="inlineStr">
+        <is>
+          <t>Analysis of the liquid sample from a catalytic test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="13" t="inlineStr">
+        <is>
+          <t>GasPhaseAnalysis</t>
+        </is>
+      </c>
+      <c r="B44" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C44" s="13" t="inlineStr">
+        <is>
+          <t>ProductIdentificationMethod</t>
+        </is>
+      </c>
+      <c r="D44" s="13" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E44" s="13" t="inlineStr"/>
+      <c r="F44" s="13" t="inlineStr"/>
+      <c r="G44" s="13" t="inlineStr"/>
+      <c r="H44" s="13" t="inlineStr"/>
+      <c r="I44" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0007814</t>
+        </is>
+      </c>
+      <c r="J44" s="13" t="inlineStr">
+        <is>
+          <t>Analysis of the liquid sample from a catalytic test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="11" t="inlineStr">
         <is>
           <t>carried out by</t>
         </is>
       </c>
-      <c r="B19" s="11" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C19" s="11" t="inlineStr"/>
-      <c r="D19" s="11" t="inlineStr">
+      <c r="B45" s="11" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C45" s="11" t="inlineStr"/>
+      <c r="D45" s="11" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="E45" s="11" t="inlineStr">
         <is>
           <t>ChemicalReactor</t>
         </is>
       </c>
-      <c r="F19" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G19" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H19" s="11" t="inlineStr"/>
-      <c r="I19" s="11" t="inlineStr"/>
-      <c r="J19" s="11" t="inlineStr">
+      <c r="F45" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G45" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H45" s="11" t="inlineStr"/>
+      <c r="I45" s="11" t="inlineStr"/>
+      <c r="J45" s="11" t="inlineStr">
         <is>
           <t>The reactor in which the Reaction takes place.
 Must be a Reactor instance (a Device subclass specific to catalytic
@@ -22761,37 +23706,37 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="13" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="13" t="inlineStr">
         <is>
           <t>ChemicalReactor</t>
         </is>
       </c>
-      <c r="B20" s="13" t="inlineStr">
+      <c r="B46" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C20" s="13" t="inlineStr">
+      <c r="C46" s="13" t="inlineStr">
         <is>
           <t>carried out by</t>
         </is>
       </c>
-      <c r="D20" s="13" t="inlineStr">
+      <c r="D46" s="13" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E20" s="13" t="inlineStr"/>
-      <c r="F20" s="13" t="inlineStr"/>
-      <c r="G20" s="13" t="inlineStr"/>
-      <c r="H20" s="13" t="inlineStr"/>
-      <c r="I20" s="13" t="inlineStr">
+      <c r="E46" s="13" t="inlineStr"/>
+      <c r="F46" s="13" t="inlineStr"/>
+      <c r="G46" s="13" t="inlineStr"/>
+      <c r="H46" s="13" t="inlineStr"/>
+      <c r="I46" s="13" t="inlineStr">
         <is>
           <t>VOC4CAT:0007018</t>
         </is>
       </c>
-      <c r="J20" s="13" t="inlineStr">
+      <c r="J46" s="13" t="inlineStr">
         <is>
           <t>Abstract Device subclass representing a catalytic reactor vessel.
 Reactor is more specific than the general Device (AgenticEntity): it restricts
@@ -22804,222 +23749,610 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="13" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="13" t="inlineStr">
         <is>
           <t>ElectrochemicalReactor</t>
         </is>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B47" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C21" s="13" t="inlineStr">
+      <c r="C47" s="13" t="inlineStr">
         <is>
           <t>ChemicalReactor</t>
         </is>
       </c>
-      <c r="D21" s="13" t="inlineStr">
+      <c r="D47" s="13" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E21" s="13" t="inlineStr"/>
-      <c r="F21" s="13" t="inlineStr"/>
-      <c r="G21" s="13" t="inlineStr"/>
-      <c r="H21" s="13" t="inlineStr"/>
-      <c r="I21" s="13" t="inlineStr">
+      <c r="E47" s="13" t="inlineStr"/>
+      <c r="F47" s="13" t="inlineStr"/>
+      <c r="G47" s="13" t="inlineStr"/>
+      <c r="H47" s="13" t="inlineStr"/>
+      <c r="I47" s="13" t="inlineStr">
         <is>
           <t>VOC4CAT:0000193</t>
         </is>
       </c>
-      <c r="J21" s="13" t="inlineStr">
+      <c r="J47" s="13" t="inlineStr">
         <is>
           <t>Electrochemical reactor used in electrocatalytic experiments, including
 H-cells, flow cells, and membrane electrode assemblies.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="13" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="12" t="inlineStr">
+        <is>
+          <t>has cathode</t>
+        </is>
+      </c>
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C48" s="12" t="inlineStr">
+        <is>
+          <t>ElectrochemicalReactor</t>
+        </is>
+      </c>
+      <c r="D48" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E48" s="12" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="F48" s="12" t="inlineStr"/>
+      <c r="G48" s="12" t="inlineStr"/>
+      <c r="H48" s="12" t="inlineStr"/>
+      <c r="I48" s="12" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0007254</t>
+        </is>
+      </c>
+      <c r="J48" s="12" t="inlineStr">
+        <is>
+          <t>The electrode where reduction occurs in an electrochemical cell. It is the negative electrode in an electrolytic cell, while it is the positive electrode in a galvanic cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="12" t="inlineStr">
+        <is>
+          <t>has anode</t>
+        </is>
+      </c>
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C49" s="12" t="inlineStr">
+        <is>
+          <t>ElectrochemicalReactor</t>
+        </is>
+      </c>
+      <c r="D49" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E49" s="12" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="F49" s="12" t="inlineStr"/>
+      <c r="G49" s="12" t="inlineStr"/>
+      <c r="H49" s="12" t="inlineStr"/>
+      <c r="I49" s="12" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0007255</t>
+        </is>
+      </c>
+      <c r="J49" s="12" t="inlineStr">
+        <is>
+          <t>The electrode where oxidation occurs in an electrochemical cell. It is the positive electrode in an electrolytic cell, while it is the negative electrode in a galvanic cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="12" t="inlineStr">
+        <is>
+          <t>has cell operating mode</t>
+        </is>
+      </c>
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C50" s="12" t="inlineStr">
+        <is>
+          <t>ElectrochemicalReactor</t>
+        </is>
+      </c>
+      <c r="D50" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E50" s="12" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="F50" s="12" t="inlineStr"/>
+      <c r="G50" s="12" t="inlineStr"/>
+      <c r="H50" s="12" t="inlineStr"/>
+      <c r="I50" s="12" t="inlineStr">
+        <is>
+          <t>SIO:000008</t>
+        </is>
+      </c>
+      <c r="J50" s="12" t="inlineStr">
+        <is>
+          <t>The functional mode of an electrochemical cell based on the direction of energy conversion, specifiying wheter the system generates electrical energy from spontaneous reactions or consumes energy to drive non-spontaneous reactions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="12" t="inlineStr">
+        <is>
+          <t>has active area</t>
+        </is>
+      </c>
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C51" s="12" t="inlineStr">
+        <is>
+          <t>ElectrochemicalReactor</t>
+        </is>
+      </c>
+      <c r="D51" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E51" s="12" t="inlineStr">
+        <is>
+          <t>QuantitativeAttribute</t>
+        </is>
+      </c>
+      <c r="F51" s="12" t="inlineStr"/>
+      <c r="G51" s="12" t="inlineStr"/>
+      <c r="H51" s="12" t="inlineStr"/>
+      <c r="I51" s="12" t="inlineStr">
+        <is>
+          <t>SIO:000008</t>
+        </is>
+      </c>
+      <c r="J51" s="12" t="inlineStr">
+        <is>
+          <t>In contrast to substrate area, the actual area of a sample or electrode which is active.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="12" t="inlineStr">
+        <is>
+          <t>has faradaic current</t>
+        </is>
+      </c>
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C52" s="12" t="inlineStr">
+        <is>
+          <t>ElectrochemicalReactor</t>
+        </is>
+      </c>
+      <c r="D52" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E52" s="12" t="inlineStr">
+        <is>
+          <t>QuantitativeAttribute</t>
+        </is>
+      </c>
+      <c r="F52" s="12" t="inlineStr"/>
+      <c r="G52" s="12" t="inlineStr"/>
+      <c r="H52" s="12" t="inlineStr"/>
+      <c r="I52" s="12" t="inlineStr">
+        <is>
+          <t>SIO:000008</t>
+        </is>
+      </c>
+      <c r="J52" s="12" t="inlineStr">
+        <is>
+          <t>The current that is flowing through an electrochemical cell and is causing (or is caused by) chemical reactions (charge transfer) occurring at the electrode surfaces.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="13" t="inlineStr">
         <is>
           <t>CSTR</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B53" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C22" s="13" t="inlineStr">
+      <c r="C53" s="13" t="inlineStr">
         <is>
           <t>ChemicalReactor</t>
         </is>
       </c>
-      <c r="D22" s="13" t="inlineStr">
+      <c r="D53" s="13" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E22" s="13" t="inlineStr"/>
-      <c r="F22" s="13" t="inlineStr"/>
-      <c r="G22" s="13" t="inlineStr"/>
-      <c r="H22" s="13" t="inlineStr"/>
-      <c r="I22" s="13" t="inlineStr">
+      <c r="E53" s="13" t="inlineStr"/>
+      <c r="F53" s="13" t="inlineStr"/>
+      <c r="G53" s="13" t="inlineStr"/>
+      <c r="H53" s="13" t="inlineStr"/>
+      <c r="I53" s="13" t="inlineStr">
         <is>
           <t>VOC4CAT:0007019</t>
         </is>
       </c>
-      <c r="J22" s="13" t="inlineStr">
+      <c r="J53" s="13" t="inlineStr">
         <is>
           <t>Continuous stirred tank reactor (CSTR) — a well-mixed, continuous-flow
 reactor operating at steady state.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="13" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="12" t="inlineStr">
+        <is>
+          <t>has stirring speed</t>
+        </is>
+      </c>
+      <c r="B54" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C54" s="12" t="inlineStr">
+        <is>
+          <t>CSTR</t>
+        </is>
+      </c>
+      <c r="D54" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E54" s="12" t="inlineStr">
+        <is>
+          <t>AngularVelocity</t>
+        </is>
+      </c>
+      <c r="F54" s="12" t="inlineStr"/>
+      <c r="G54" s="12" t="inlineStr"/>
+      <c r="H54" s="12" t="inlineStr"/>
+      <c r="I54" s="12" t="inlineStr">
+        <is>
+          <t>SIO:000008</t>
+        </is>
+      </c>
+      <c r="J54" s="12" t="inlineStr">
+        <is>
+          <t>Rotational speed of stirring or agitation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="13" t="inlineStr">
+        <is>
+          <t>AngularVelocity</t>
+        </is>
+      </c>
+      <c r="B55" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C55" s="13" t="inlineStr">
+        <is>
+          <t>has stirring speed</t>
+        </is>
+      </c>
+      <c r="D55" s="13" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E55" s="13" t="inlineStr"/>
+      <c r="F55" s="13" t="inlineStr"/>
+      <c r="G55" s="13" t="inlineStr"/>
+      <c r="H55" s="13" t="inlineStr"/>
+      <c r="I55" s="13" t="inlineStr">
+        <is>
+          <t>qudt:Quantity</t>
+        </is>
+      </c>
+      <c r="J55" s="13" t="inlineStr">
+        <is>
+          <t>Rate of rotational motion, typically expressed in revolutions per minute.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="12" t="inlineStr">
+        <is>
+          <t>has volume</t>
+        </is>
+      </c>
+      <c r="B56" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C56" s="12" t="inlineStr">
+        <is>
+          <t>CSTR</t>
+        </is>
+      </c>
+      <c r="D56" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E56" s="12" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="F56" s="12" t="inlineStr"/>
+      <c r="G56" s="12" t="inlineStr"/>
+      <c r="H56" s="12" t="inlineStr"/>
+      <c r="I56" s="12" t="inlineStr"/>
+      <c r="J56" s="12" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="12" t="inlineStr">
+        <is>
+          <t>has stirrer type</t>
+        </is>
+      </c>
+      <c r="B57" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C57" s="12" t="inlineStr">
+        <is>
+          <t>CSTR</t>
+        </is>
+      </c>
+      <c r="D57" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E57" s="12" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="F57" s="12" t="inlineStr"/>
+      <c r="G57" s="12" t="inlineStr"/>
+      <c r="H57" s="12" t="inlineStr"/>
+      <c r="I57" s="12" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0008113</t>
+        </is>
+      </c>
+      <c r="J57" s="12" t="inlineStr">
+        <is>
+          <t>The category of mechanical or magnetic agitation device used to ensure homogeneous mixing within a reaction system or mixing vessel, such as a magnetic stirrer or an overhead mechanical (steel shaft) stirrer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="12" t="inlineStr">
+        <is>
+          <t>has stirrer diameter</t>
+        </is>
+      </c>
+      <c r="B58" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C58" s="12" t="inlineStr">
+        <is>
+          <t>CSTR</t>
+        </is>
+      </c>
+      <c r="D58" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E58" s="12" t="inlineStr">
+        <is>
+          <t>QuantitativeAttribute</t>
+        </is>
+      </c>
+      <c r="F58" s="12" t="inlineStr"/>
+      <c r="G58" s="12" t="inlineStr"/>
+      <c r="H58" s="12" t="inlineStr"/>
+      <c r="I58" s="12" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0008115</t>
+        </is>
+      </c>
+      <c r="J58" s="12" t="inlineStr">
+        <is>
+          <t>The effective diameter of the stirrer. Typically expressed as the distance across the rotating blade or mixing head from one tip to the opposite tip.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="13" t="inlineStr">
         <is>
           <t>PlugFlowReactor</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B59" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C23" s="13" t="inlineStr">
+      <c r="C59" s="13" t="inlineStr">
         <is>
           <t>ChemicalReactor</t>
         </is>
       </c>
-      <c r="D23" s="13" t="inlineStr">
+      <c r="D59" s="13" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E23" s="13" t="inlineStr"/>
-      <c r="F23" s="13" t="inlineStr"/>
-      <c r="G23" s="13" t="inlineStr"/>
-      <c r="H23" s="13" t="inlineStr"/>
-      <c r="I23" s="13" t="inlineStr">
+      <c r="E59" s="13" t="inlineStr"/>
+      <c r="F59" s="13" t="inlineStr"/>
+      <c r="G59" s="13" t="inlineStr"/>
+      <c r="H59" s="13" t="inlineStr"/>
+      <c r="I59" s="13" t="inlineStr">
         <is>
           <t>VOC4CAT:0007102</t>
         </is>
       </c>
-      <c r="J23" s="13" t="inlineStr">
+      <c r="J59" s="13" t="inlineStr">
         <is>
           <t>Plug flow reactor (PFR) — a tubular reactor in which reactant composition
 varies along the axis with no axial mixing.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="13" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="13" t="inlineStr">
         <is>
           <t>Autoclave</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B60" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C24" s="13" t="inlineStr">
+      <c r="C60" s="13" t="inlineStr">
         <is>
           <t>ChemicalReactor</t>
         </is>
       </c>
-      <c r="D24" s="13" t="inlineStr">
+      <c r="D60" s="13" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E24" s="13" t="inlineStr"/>
-      <c r="F24" s="13" t="inlineStr"/>
-      <c r="G24" s="13" t="inlineStr"/>
-      <c r="H24" s="13" t="inlineStr"/>
-      <c r="I24" s="13" t="inlineStr">
+      <c r="E60" s="13" t="inlineStr"/>
+      <c r="F60" s="13" t="inlineStr"/>
+      <c r="G60" s="13" t="inlineStr"/>
+      <c r="H60" s="13" t="inlineStr"/>
+      <c r="I60" s="13" t="inlineStr">
         <is>
           <t>NCIT:C93052</t>
         </is>
       </c>
-      <c r="J24" s="13" t="inlineStr">
+      <c r="J60" s="13" t="inlineStr">
         <is>
           <t>Autoclave reactor — a sealed pressure vessel for batch reactions at
 elevated temperature and/or pressure.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="13" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="13" t="inlineStr">
         <is>
           <t>SlurryReactor</t>
         </is>
       </c>
-      <c r="B25" s="13" t="inlineStr">
+      <c r="B61" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C25" s="13" t="inlineStr">
+      <c r="C61" s="13" t="inlineStr">
         <is>
           <t>ChemicalReactor</t>
         </is>
       </c>
-      <c r="D25" s="13" t="inlineStr">
+      <c r="D61" s="13" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E25" s="13" t="inlineStr"/>
-      <c r="F25" s="13" t="inlineStr"/>
-      <c r="G25" s="13" t="inlineStr"/>
-      <c r="H25" s="13" t="inlineStr"/>
-      <c r="I25" s="13" t="inlineStr">
+      <c r="E61" s="13" t="inlineStr"/>
+      <c r="F61" s="13" t="inlineStr"/>
+      <c r="G61" s="13" t="inlineStr"/>
+      <c r="H61" s="13" t="inlineStr"/>
+      <c r="I61" s="13" t="inlineStr">
         <is>
           <t>coremeta4cat:SlurryReactor</t>
         </is>
       </c>
-      <c r="J25" s="13" t="inlineStr">
+      <c r="J61" s="13" t="inlineStr">
         <is>
           <t>Slurry reactor — a three-phase reactor in which catalyst particles are
 suspended in a liquid phase through which gas is bubbled.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="13" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="13" t="inlineStr">
         <is>
           <t>Microreactor</t>
         </is>
       </c>
-      <c r="B26" s="13" t="inlineStr">
+      <c r="B62" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C26" s="13" t="inlineStr">
+      <c r="C62" s="13" t="inlineStr">
         <is>
           <t>ChemicalReactor</t>
         </is>
       </c>
-      <c r="D26" s="13" t="inlineStr">
+      <c r="D62" s="13" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E26" s="13" t="inlineStr"/>
-      <c r="F26" s="13" t="inlineStr"/>
-      <c r="G26" s="13" t="inlineStr"/>
-      <c r="H26" s="13" t="inlineStr"/>
-      <c r="I26" s="13" t="inlineStr">
+      <c r="E62" s="13" t="inlineStr"/>
+      <c r="F62" s="13" t="inlineStr"/>
+      <c r="G62" s="13" t="inlineStr"/>
+      <c r="H62" s="13" t="inlineStr"/>
+      <c r="I62" s="13" t="inlineStr">
         <is>
           <t>VOC4CAT:0000234</t>
         </is>
       </c>
-      <c r="J26" s="13" t="inlineStr">
+      <c r="J62" s="13" t="inlineStr">
         <is>
           <t>Microreactor — a miniaturised flow reactor with characteristic dimensions
 in the sub-millimetre range, enabling precise thermal control and rapid
@@ -23027,207 +24360,367 @@
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="13" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="13" t="inlineStr">
         <is>
           <t>FixedBedReactor</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B63" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C27" s="13" t="inlineStr">
+      <c r="C63" s="13" t="inlineStr">
         <is>
           <t>ChemicalReactor</t>
         </is>
       </c>
-      <c r="D27" s="13" t="inlineStr">
+      <c r="D63" s="13" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E27" s="13" t="inlineStr"/>
-      <c r="F27" s="13" t="inlineStr"/>
-      <c r="G27" s="13" t="inlineStr"/>
-      <c r="H27" s="13" t="inlineStr"/>
-      <c r="I27" s="13" t="inlineStr">
+      <c r="E63" s="13" t="inlineStr"/>
+      <c r="F63" s="13" t="inlineStr"/>
+      <c r="G63" s="13" t="inlineStr"/>
+      <c r="H63" s="13" t="inlineStr"/>
+      <c r="I63" s="13" t="inlineStr">
         <is>
           <t>coremeta4cat:FixedBedReactor</t>
         </is>
       </c>
-      <c r="J27" s="13" t="inlineStr">
+      <c r="J63" s="13" t="inlineStr">
         <is>
           <t>Fixed bed reactor — a tubular reactor packed with a stationary catalyst bed.
 The most common reactor type in heterogeneous catalysis testing.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="13" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="12" t="inlineStr">
+        <is>
+          <t>has catalyst particle size</t>
+        </is>
+      </c>
+      <c r="B64" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C64" s="12" t="inlineStr">
+        <is>
+          <t>FixedBedReactor</t>
+        </is>
+      </c>
+      <c r="D64" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E64" s="12" t="inlineStr">
+        <is>
+          <t>QuantitativeAttribute</t>
+        </is>
+      </c>
+      <c r="F64" s="12" t="inlineStr"/>
+      <c r="G64" s="12" t="inlineStr"/>
+      <c r="H64" s="12" t="inlineStr"/>
+      <c r="I64" s="12" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0008212</t>
+        </is>
+      </c>
+      <c r="J64" s="12" t="inlineStr">
+        <is>
+          <t>A measure of the characteristic linear dimension of a particle in a sample, typically reported as diameter, equivalent diameter, or another size metric determined by an appropriate measurement method.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="12" t="inlineStr">
+        <is>
+          <t>has catalyst bed volume</t>
+        </is>
+      </c>
+      <c r="B65" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C65" s="12" t="inlineStr">
+        <is>
+          <t>FixedBedReactor</t>
+        </is>
+      </c>
+      <c r="D65" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E65" s="12" t="inlineStr">
+        <is>
+          <t>QuantitativeAttribute</t>
+        </is>
+      </c>
+      <c r="F65" s="12" t="inlineStr"/>
+      <c r="G65" s="12" t="inlineStr"/>
+      <c r="H65" s="12" t="inlineStr"/>
+      <c r="I65" s="12" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0007021</t>
+        </is>
+      </c>
+      <c r="J65" s="12" t="inlineStr">
+        <is>
+          <t>The bulk volume taken up by the catalyst and potential diluent in a fixed bed reactor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="12" t="inlineStr">
+        <is>
+          <t>has catalyst dilution material</t>
+        </is>
+      </c>
+      <c r="B66" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C66" s="12" t="inlineStr">
+        <is>
+          <t>FixedBedReactor</t>
+        </is>
+      </c>
+      <c r="D66" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E66" s="12" t="inlineStr">
+        <is>
+          <t>QualitativeAttribute</t>
+        </is>
+      </c>
+      <c r="F66" s="12" t="inlineStr"/>
+      <c r="G66" s="12" t="inlineStr"/>
+      <c r="H66" s="12" t="inlineStr"/>
+      <c r="I66" s="12" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0008218</t>
+        </is>
+      </c>
+      <c r="J66" s="12" t="inlineStr">
+        <is>
+          <t>An inert solid mixed with catalyst particles in a fixed bed to modify bed properties (e.g., improve heat transfer, hydrodynamics or isothermicity) without participating in the reaction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="12" t="inlineStr">
+        <is>
+          <t>has catalyst bed height</t>
+        </is>
+      </c>
+      <c r="B67" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C67" s="12" t="inlineStr">
+        <is>
+          <t>FixedBedReactor</t>
+        </is>
+      </c>
+      <c r="D67" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E67" s="12" t="inlineStr">
+        <is>
+          <t>QuantitativeAttribute</t>
+        </is>
+      </c>
+      <c r="F67" s="12" t="inlineStr"/>
+      <c r="G67" s="12" t="inlineStr"/>
+      <c r="H67" s="12" t="inlineStr"/>
+      <c r="I67" s="12" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0008217</t>
+        </is>
+      </c>
+      <c r="J67" s="12" t="inlineStr">
+        <is>
+          <t>The axial length of the packed catalyst section in a reactor, measured along the direction of flow between the defined bed boundaries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="13" t="inlineStr">
         <is>
           <t>FluidizedBedReactor</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="B68" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C28" s="13" t="inlineStr">
+      <c r="C68" s="13" t="inlineStr">
         <is>
           <t>ChemicalReactor</t>
         </is>
       </c>
-      <c r="D28" s="13" t="inlineStr">
+      <c r="D68" s="13" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E28" s="13" t="inlineStr"/>
-      <c r="F28" s="13" t="inlineStr"/>
-      <c r="G28" s="13" t="inlineStr"/>
-      <c r="H28" s="13" t="inlineStr"/>
-      <c r="I28" s="13" t="inlineStr">
+      <c r="E68" s="13" t="inlineStr"/>
+      <c r="F68" s="13" t="inlineStr"/>
+      <c r="G68" s="13" t="inlineStr"/>
+      <c r="H68" s="13" t="inlineStr"/>
+      <c r="I68" s="13" t="inlineStr">
         <is>
           <t>coremeta4cat:FluidizedBedReactor</t>
         </is>
       </c>
-      <c r="J28" s="13" t="inlineStr">
+      <c r="J68" s="13" t="inlineStr">
         <is>
           <t>Fluidized bed reactor — a reactor in which the catalyst particles are
 suspended in an upward-flowing gas or liquid stream.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="12" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="12" t="inlineStr">
         <is>
           <t>gas distributor type</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C29" s="12" t="inlineStr">
+      <c r="B69" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C69" s="12" t="inlineStr">
         <is>
           <t>FluidizedBedReactor</t>
         </is>
       </c>
-      <c r="D29" s="12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E29" s="12" t="inlineStr">
+      <c r="D69" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E69" s="12" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="F29" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G29" s="12" t="inlineStr"/>
-      <c r="H29" s="12" t="inlineStr"/>
-      <c r="I29" s="12" t="inlineStr">
+      <c r="F69" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G69" s="12" t="inlineStr"/>
+      <c r="H69" s="12" t="inlineStr"/>
+      <c r="I69" s="12" t="inlineStr">
         <is>
           <t>coremeta4cat:gas_distributor_type</t>
         </is>
       </c>
-      <c r="J29" s="12" t="inlineStr">
+      <c r="J69" s="12" t="inlineStr">
         <is>
           <t>Type or design of the gas distributor plate in a fluidized bed reactor.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="12" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="12" t="inlineStr">
         <is>
           <t>bed expansion height</t>
         </is>
       </c>
-      <c r="B30" s="12" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C30" s="12" t="inlineStr">
+      <c r="B70" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C70" s="12" t="inlineStr">
         <is>
           <t>FluidizedBedReactor</t>
         </is>
       </c>
-      <c r="D30" s="12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E30" s="12" t="inlineStr">
+      <c r="D70" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E70" s="12" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="F30" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G30" s="12" t="inlineStr"/>
-      <c r="H30" s="12" t="inlineStr">
+      <c r="F70" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G70" s="12" t="inlineStr"/>
+      <c r="H70" s="12" t="inlineStr">
         <is>
           <t>cm</t>
         </is>
       </c>
-      <c r="I30" s="12" t="inlineStr">
+      <c r="I70" s="12" t="inlineStr">
         <is>
           <t>coremeta4cat:bed_expansion_height</t>
         </is>
       </c>
-      <c r="J30" s="12" t="inlineStr">
+      <c r="J70" s="12" t="inlineStr">
         <is>
           <t>Height of bed expansion above the settled bed height under operating conditions.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="12" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="12" t="inlineStr">
         <is>
           <t>bubble size distribution</t>
         </is>
       </c>
-      <c r="B31" s="12" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C31" s="12" t="inlineStr">
+      <c r="B71" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C71" s="12" t="inlineStr">
         <is>
           <t>FluidizedBedReactor</t>
         </is>
       </c>
-      <c r="D31" s="12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E31" s="12" t="inlineStr">
+      <c r="D71" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E71" s="12" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="F31" s="12" t="inlineStr"/>
-      <c r="G31" s="12" t="inlineStr"/>
-      <c r="H31" s="12" t="inlineStr"/>
-      <c r="I31" s="12" t="inlineStr">
+      <c r="F71" s="12" t="inlineStr"/>
+      <c r="G71" s="12" t="inlineStr"/>
+      <c r="H71" s="12" t="inlineStr"/>
+      <c r="I71" s="12" t="inlineStr">
         <is>
           <t>coremeta4cat:bubble_size_distribution</t>
         </is>
       </c>
-      <c r="J31" s="12" t="inlineStr">
+      <c r="J71" s="12" t="inlineStr">
         <is>
           <t>Description or characterization of bubble size distribution in the fluidized bed.</t>
         </is>

</xml_diff>